<commit_message>
Update travel certificate templates and generation
</commit_message>
<xml_diff>
--- a/PROJECTS/Documents/2. DocumentsGeneration/Results/Квитки.xlsx
+++ b/PROJECTS/Documents/2. DocumentsGeneration/Results/Квитки.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="Workbook________" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\Excel\PROJECTS\2. DocumentsGeneration\Results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS\Documents\2. DocumentsGeneration\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00A2CF3A-9914-4671-8CDB-1CF0055B44E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA97AC9-6033-4D14-A1FA-179F18EA01DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FF16710E-FAF6-445F-AD75-CD3560A0E894}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Звання</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>Статус</t>
+  </si>
+  <si>
+    <t>Куди</t>
   </si>
 </sst>
 </file>
@@ -210,7 +213,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -290,12 +293,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -359,6 +373,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -366,7 +383,81 @@
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
     <cellStyle name="Обычный 4" xfId="1" xr:uid="{98265266-0594-4C2A-BAC9-F7BD39857057}"/>
   </cellStyles>
-  <dxfs count="33">
+  <dxfs count="34">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="4" tint="0.39997558519241921"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1170,39 +1261,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="1" tint="0.249977111117893"/>
@@ -1308,14 +1366,14 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="TableStyleDark_my" pivot="0" count="8" xr9:uid="{CFC3E1FC-0CEF-4FBB-AEF8-B86D335BF785}">
-      <tableStyleElement type="wholeTable" dxfId="32"/>
-      <tableStyleElement type="headerRow" dxfId="31"/>
-      <tableStyleElement type="totalRow" dxfId="30"/>
-      <tableStyleElement type="firstColumn" dxfId="29"/>
-      <tableStyleElement type="lastColumn" dxfId="28"/>
-      <tableStyleElement type="firstRowStripe" dxfId="27"/>
-      <tableStyleElement type="secondRowStripe" dxfId="26"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="25"/>
+      <tableStyleElement type="wholeTable" dxfId="33"/>
+      <tableStyleElement type="headerRow" dxfId="32"/>
+      <tableStyleElement type="totalRow" dxfId="31"/>
+      <tableStyleElement type="firstColumn" dxfId="30"/>
+      <tableStyleElement type="lastColumn" dxfId="29"/>
+      <tableStyleElement type="firstRowStripe" dxfId="28"/>
+      <tableStyleElement type="secondRowStripe" dxfId="27"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="26"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1330,28 +1388,29 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8633DC14-6705-4E28-96A1-2100186D89C1}" name="tbTickets" displayName="tbTickets" ref="C3:U4" totalsRowShown="0" headerRowDxfId="24" dataDxfId="22" headerRowBorderDxfId="23" tableBorderDxfId="21" totalsRowBorderDxfId="20">
-  <autoFilter ref="C3:U4" xr:uid="{8633DC14-6705-4E28-96A1-2100186D89C1}"/>
-  <tableColumns count="19">
-    <tableColumn id="15" xr3:uid="{1248187E-92DC-48D8-9F19-B3F422FC96EE}" name="Звання" dataDxfId="19" dataCellStyle="Обычный 4"/>
-    <tableColumn id="14" xr3:uid="{8DD6B219-3207-45AE-A047-947A65847ECC}" name="ПІБ" dataDxfId="18" dataCellStyle="Обычный 4"/>
-    <tableColumn id="12" xr3:uid="{F4B0E700-28E8-4F8D-8D4B-560C462D4E10}" name="ІПН" dataDxfId="17" dataCellStyle="Обычный 4"/>
-    <tableColumn id="1" xr3:uid="{18FCA8B5-D94E-49E1-8486-281C0C59574E}" name="Посада" dataDxfId="16" dataCellStyle="Обычный 4"/>
-    <tableColumn id="6" xr3:uid="{E06CAB9E-9045-46C0-9E50-D811A3F3E047}" name="Подія" dataDxfId="15" dataCellStyle="Обычный 4"/>
-    <tableColumn id="4" xr3:uid="{1B3E7AFC-25CB-4E78-9DB2-F81AFB13D0FE}" name="Вибуття.Наказ" dataDxfId="14" dataCellStyle="Обычный 4"/>
-    <tableColumn id="2" xr3:uid="{45B6644A-F362-4997-82ED-3840673FBB21}" name="Вибуття.Продовольче" dataDxfId="13" dataCellStyle="Обычный 4"/>
-    <tableColumn id="3" xr3:uid="{17E6962A-CD97-4A63-88C5-3EDCAC7FCA4A}" name="Вибуття" dataDxfId="12" dataCellStyle="Обычный 4"/>
-    <tableColumn id="5" xr3:uid="{D5916072-D2BF-42E4-AC0E-C0D107F9C492}" name="Вибуття.Термін" dataDxfId="11" dataCellStyle="Обычный 4"/>
-    <tableColumn id="7" xr3:uid="{F607D590-8EA4-4671-9BB9-DB68458A2134}" name="Вибуття.Дорога" dataDxfId="10" dataCellStyle="Обычный 4"/>
-    <tableColumn id="8" xr3:uid="{B504EEBB-4C9B-46FA-832A-257F577794EE}" name="Прибуття.План" dataDxfId="9" dataCellStyle="Обычный 4"/>
-    <tableColumn id="9" xr3:uid="{ACEDC157-4114-4FED-8A66-B9F13885F0DF}" name="Прибуття" dataDxfId="8" dataCellStyle="Обычный 4"/>
-    <tableColumn id="10" xr3:uid="{C0246A93-DF0E-4E98-A206-6EB398B6649F}" name="Прибуття.Продовольче" dataDxfId="7" dataCellStyle="Обычный 4"/>
-    <tableColumn id="11" xr3:uid="{3DFAB9D4-EF74-4118-AD75-62B4C8EEC570}" name="Прибуття.Наказ" dataDxfId="6" dataCellStyle="Обычный 4"/>
-    <tableColumn id="13" xr3:uid="{3EAA7D42-1DA5-425D-B5C5-177178CD4DAB}" name="Супровідний документ" dataDxfId="5" dataCellStyle="Обычный 4"/>
-    <tableColumn id="17" xr3:uid="{B7D8EDE7-1D3B-48AB-BC35-5A54DAE16C6B}" name="ТВО.ПІБ" dataDxfId="4" dataCellStyle="Обычный 4"/>
-    <tableColumn id="18" xr3:uid="{40D6D168-F077-46FE-AC0E-8FB87005760B}" name="ТВО.ІПН" dataDxfId="3" dataCellStyle="Обычный 4"/>
-    <tableColumn id="19" xr3:uid="{EFBB7D0E-414E-4CA7-BB9E-52B50136B5AE}" name="ТВО.Посада" dataDxfId="2" dataCellStyle="Обычный 4"/>
-    <tableColumn id="16" xr3:uid="{EF1450E4-A6A7-43BA-8551-213C379B6E96}" name="Статус" dataDxfId="1" dataCellStyle="Обычный 4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8633DC14-6705-4E28-96A1-2100186D89C1}" name="tbTickets" displayName="tbTickets" ref="C3:V4" totalsRowShown="0" headerRowDxfId="1" dataDxfId="25" headerRowBorderDxfId="2" tableBorderDxfId="24" totalsRowBorderDxfId="23">
+  <autoFilter ref="C3:V4" xr:uid="{8633DC14-6705-4E28-96A1-2100186D89C1}"/>
+  <tableColumns count="20">
+    <tableColumn id="15" xr3:uid="{1248187E-92DC-48D8-9F19-B3F422FC96EE}" name="Звання" dataDxfId="22" dataCellStyle="Обычный 4"/>
+    <tableColumn id="14" xr3:uid="{8DD6B219-3207-45AE-A047-947A65847ECC}" name="ПІБ" dataDxfId="21" dataCellStyle="Обычный 4"/>
+    <tableColumn id="12" xr3:uid="{F4B0E700-28E8-4F8D-8D4B-560C462D4E10}" name="ІПН" dataDxfId="20" dataCellStyle="Обычный 4"/>
+    <tableColumn id="1" xr3:uid="{18FCA8B5-D94E-49E1-8486-281C0C59574E}" name="Посада" dataDxfId="19" dataCellStyle="Обычный 4"/>
+    <tableColumn id="6" xr3:uid="{E06CAB9E-9045-46C0-9E50-D811A3F3E047}" name="Подія" dataDxfId="18" dataCellStyle="Обычный 4"/>
+    <tableColumn id="4" xr3:uid="{1B3E7AFC-25CB-4E78-9DB2-F81AFB13D0FE}" name="Куди" dataDxfId="17" dataCellStyle="Обычный 4"/>
+    <tableColumn id="2" xr3:uid="{45B6644A-F362-4997-82ED-3840673FBB21}" name="Вибуття.Наказ" dataDxfId="16" dataCellStyle="Обычный 4"/>
+    <tableColumn id="3" xr3:uid="{17E6962A-CD97-4A63-88C5-3EDCAC7FCA4A}" name="Вибуття.Продовольче" dataDxfId="15" dataCellStyle="Обычный 4"/>
+    <tableColumn id="5" xr3:uid="{D5916072-D2BF-42E4-AC0E-C0D107F9C492}" name="Вибуття" dataDxfId="14" dataCellStyle="Обычный 4"/>
+    <tableColumn id="7" xr3:uid="{F607D590-8EA4-4671-9BB9-DB68458A2134}" name="Вибуття.Термін" dataDxfId="13" dataCellStyle="Обычный 4"/>
+    <tableColumn id="8" xr3:uid="{B504EEBB-4C9B-46FA-832A-257F577794EE}" name="Вибуття.Дорога" dataDxfId="12" dataCellStyle="Обычный 4"/>
+    <tableColumn id="9" xr3:uid="{ACEDC157-4114-4FED-8A66-B9F13885F0DF}" name="Прибуття.План" dataDxfId="11" dataCellStyle="Обычный 4"/>
+    <tableColumn id="10" xr3:uid="{C0246A93-DF0E-4E98-A206-6EB398B6649F}" name="Прибуття" dataDxfId="10" dataCellStyle="Обычный 4"/>
+    <tableColumn id="11" xr3:uid="{3DFAB9D4-EF74-4118-AD75-62B4C8EEC570}" name="Прибуття.Продовольче" dataDxfId="9" dataCellStyle="Обычный 4"/>
+    <tableColumn id="13" xr3:uid="{3EAA7D42-1DA5-425D-B5C5-177178CD4DAB}" name="Прибуття.Наказ" dataDxfId="8" dataCellStyle="Обычный 4"/>
+    <tableColumn id="17" xr3:uid="{B7D8EDE7-1D3B-48AB-BC35-5A54DAE16C6B}" name="Супровідний документ" dataDxfId="7" dataCellStyle="Обычный 4"/>
+    <tableColumn id="18" xr3:uid="{40D6D168-F077-46FE-AC0E-8FB87005760B}" name="ТВО.ПІБ" dataDxfId="6" dataCellStyle="Обычный 4"/>
+    <tableColumn id="19" xr3:uid="{EFBB7D0E-414E-4CA7-BB9E-52B50136B5AE}" name="ТВО.ІПН" dataDxfId="5" dataCellStyle="Обычный 4"/>
+    <tableColumn id="16" xr3:uid="{EF1450E4-A6A7-43BA-8551-213C379B6E96}" name="ТВО.Посада" dataDxfId="4" dataCellStyle="Обычный 4"/>
+    <tableColumn id="20" xr3:uid="{0A49030C-204A-48C9-B014-525F669DD949}" name="Статус" dataDxfId="0" dataCellStyle="Обычный 4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark_my" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1684,20 +1743,20 @@
     <col min="4" max="4" width="26.625" style="1" customWidth="1"/>
     <col min="5" max="5" width="17" style="1" customWidth="1"/>
     <col min="6" max="6" width="20.75" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.75" style="1" customWidth="1"/>
-    <col min="10" max="10" width="11.875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9" style="1" customWidth="1"/>
-    <col min="12" max="12" width="9.125" style="1" customWidth="1"/>
-    <col min="13" max="15" width="11.875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="10.125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="14.375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="14" style="1" customWidth="1"/>
-    <col min="19" max="19" width="15.375" style="1" customWidth="1"/>
-    <col min="20" max="20" width="19.75" style="1" customWidth="1"/>
-    <col min="21" max="21" width="17.625" style="1" customWidth="1"/>
-    <col min="22" max="16384" width="9" style="1"/>
+    <col min="7" max="8" width="16.625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="9" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.75" style="1" customWidth="1"/>
+    <col min="11" max="11" width="11.875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9" style="1" customWidth="1"/>
+    <col min="13" max="13" width="9.125" style="1" customWidth="1"/>
+    <col min="14" max="16" width="11.875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="10.125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="14.375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="14" style="1" customWidth="1"/>
+    <col min="20" max="20" width="15.375" style="1" customWidth="1"/>
+    <col min="21" max="21" width="19.75" style="1" customWidth="1"/>
+    <col min="22" max="22" width="17.625" style="1" customWidth="1"/>
+    <col min="23" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:22" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -1722,46 +1781,49 @@
       <c r="G3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="K3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="L3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="6" t="s">
+      <c r="M3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="M3" s="11" t="s">
+      <c r="N3" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="N3" s="11" t="s">
+      <c r="O3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="O3" s="11" t="s">
+      <c r="P3" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="P3" s="12" t="s">
+      <c r="Q3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="Q3" s="12" t="s">
+      <c r="R3" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="R3" s="11" t="s">
+      <c r="S3" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="S3" s="11" t="s">
+      <c r="T3" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="T3" s="12" t="s">
+      <c r="U3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="U3" s="12" t="s">
+      <c r="V3" s="12" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1779,7 +1841,7 @@
       <c r="K4" s="19"/>
       <c r="L4" s="19"/>
       <c r="M4" s="20" t="str">
-        <f>IF(0&lt;LEN(tbTickets[[#This Row],[Вибуття.Термін]]),tbTickets[[#This Row],[Вибуття]]+SUM(tbTickets[[#This Row],[Вибуття.Термін]],tbTickets[[#This Row],[Вибуття.Дорога]]),"")</f>
+        <f>IF(0&lt;LEN(tbTickets[[#This Row],[Вибуття]]),tbTickets[[#This Row],[Вибуття.Продовольче]]+SUM(tbTickets[[#This Row],[Вибуття]],tbTickets[[#This Row],[Вибуття.Термін]]),"")</f>
         <v/>
       </c>
       <c r="N4" s="21"/>
@@ -1790,12 +1852,12 @@
       <c r="S4" s="13"/>
       <c r="T4" s="13"/>
       <c r="U4" s="22"/>
-      <c r="V4" s="2"/>
+      <c r="V4" s="23"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="D4">
-    <cfRule type="duplicateValues" dxfId="0" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="33"/>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4" xr:uid="{DFEFF6E8-FDB7-4076-B447-2C0F4B46CE62}">

</xml_diff>